<commit_message>
feat(data): nouvelle mise à jour listes joueurs A et B
</commit_message>
<xml_diff>
--- a/public/data/@LISTE  GROUPE A.xlsx
+++ b/public/data/@LISTE  GROUPE A.xlsx
@@ -28765,8 +28765,8 @@
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="20">
-        <v>26.0</v>
+      <c r="A33" s="59">
+        <v>1.0</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>22</v>

</xml_diff>